<commit_message>
Weights sheet: use storefront product links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GZ6mf45gFCeDpGL3ireK6C
</commit_message>
<xml_diff>
--- a/docs/Bhoomija_Weights_Needed.xlsx
+++ b/docs/Bhoomija_Weights_Needed.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -60,10 +64,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,7 +443,7 @@
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,7 +479,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Admin link</t>
+          <t>Product link</t>
         </is>
       </c>
     </row>
@@ -501,9 +506,9 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496618668079</t>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-kauna-u-bag</t>
         </is>
       </c>
     </row>
@@ -530,9 +535,9 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660774959</t>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-u-bag</t>
         </is>
       </c>
     </row>
@@ -559,9 +564,9 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660807727</t>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-bag</t>
         </is>
       </c>
     </row>
@@ -588,9 +593,9 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496647307311</t>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-water-hyacinth-bag</t>
         </is>
       </c>
     </row>
@@ -617,9 +622,9 @@
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496661102639</t>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kauna-cherry-bag-with-bhoomija-logo</t>
         </is>
       </c>
     </row>
@@ -646,9 +651,9 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643276847</t>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-belt-brown</t>
         </is>
       </c>
     </row>
@@ -679,9 +684,9 @@
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk</t>
         </is>
       </c>
     </row>
@@ -712,9 +717,9 @@
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk</t>
         </is>
       </c>
     </row>
@@ -745,9 +750,9 @@
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk</t>
         </is>
       </c>
     </row>
@@ -778,9 +783,9 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk</t>
         </is>
       </c>
     </row>
@@ -811,9 +816,9 @@
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk</t>
         </is>
       </c>
     </row>
@@ -844,9 +849,9 @@
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk</t>
         </is>
       </c>
     </row>
@@ -877,9 +882,9 @@
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk</t>
         </is>
       </c>
     </row>
@@ -910,9 +915,9 @@
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496647077935</t>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/embroidered-moon-clutch-waterhyacinth</t>
         </is>
       </c>
     </row>
@@ -943,9 +948,9 @@
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496647077935</t>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/embroidered-moon-clutch-waterhyacinth</t>
         </is>
       </c>
     </row>
@@ -976,9 +981,9 @@
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496661135407</t>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroirdered-kauna-moon-clutch</t>
         </is>
       </c>
     </row>
@@ -1009,9 +1014,9 @@
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496661135407</t>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroirdered-kauna-moon-clutch</t>
         </is>
       </c>
     </row>
@@ -1038,9 +1043,9 @@
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496618602543</t>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kauna-purse-white-flower-with-green-leaves</t>
         </is>
       </c>
     </row>
@@ -1071,9 +1076,9 @@
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496655368239</t>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-clutch-purse</t>
         </is>
       </c>
     </row>
@@ -1104,9 +1109,9 @@
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496655368239</t>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-clutch-purse</t>
         </is>
       </c>
     </row>
@@ -1137,9 +1142,9 @@
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496653926447</t>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-handpainted-clutch-bag</t>
         </is>
       </c>
     </row>
@@ -1170,9 +1175,9 @@
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496653926447</t>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-handpainted-clutch-bag</t>
         </is>
       </c>
     </row>
@@ -1203,9 +1208,9 @@
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496653926447</t>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-handpainted-clutch-bag</t>
         </is>
       </c>
     </row>
@@ -1232,9 +1237,9 @@
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496647143471</t>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/plain-moon-clutch-waterhyacinth</t>
         </is>
       </c>
     </row>
@@ -1261,9 +1266,9 @@
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496647241775</t>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/water-hyacinth-handbag</t>
         </is>
       </c>
     </row>
@@ -1294,9 +1299,9 @@
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641835055</t>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sohrai-11-by-15</t>
         </is>
       </c>
     </row>
@@ -1327,9 +1332,9 @@
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641835055</t>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sohrai-11-by-15</t>
         </is>
       </c>
     </row>
@@ -1360,9 +1365,9 @@
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641835055</t>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sohrai-11-by-15</t>
         </is>
       </c>
     </row>
@@ -1389,9 +1394,9 @@
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496656056367</t>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframed-makhana-making-sujani-embroidery-in-process</t>
         </is>
       </c>
     </row>
@@ -1418,9 +1423,9 @@
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660054063</t>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single</t>
         </is>
       </c>
     </row>
@@ -1447,9 +1452,9 @@
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660119599</t>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-1</t>
         </is>
       </c>
     </row>
@@ -1476,9 +1481,9 @@
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660217903</t>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-2</t>
         </is>
       </c>
     </row>
@@ -1505,9 +1510,9 @@
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660250671</t>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-3</t>
         </is>
       </c>
     </row>
@@ -1534,9 +1539,9 @@
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660283439</t>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-4</t>
         </is>
       </c>
     </row>
@@ -1563,9 +1568,9 @@
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660316207</t>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-5</t>
         </is>
       </c>
     </row>
@@ -1592,9 +1597,9 @@
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659857455</t>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bedspread-king</t>
         </is>
       </c>
     </row>
@@ -1621,9 +1626,9 @@
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659890223</t>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bedspread-king-1</t>
         </is>
       </c>
     </row>
@@ -1650,9 +1655,9 @@
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659922991</t>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bedspread-king-2</t>
         </is>
       </c>
     </row>
@@ -1679,9 +1684,9 @@
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659955759</t>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bed-spread-queen</t>
         </is>
       </c>
     </row>
@@ -1708,9 +1713,9 @@
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659988527</t>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bed-spread-queen-1</t>
         </is>
       </c>
     </row>
@@ -1737,9 +1742,9 @@
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660021295</t>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bed-spread-queen-2</t>
         </is>
       </c>
     </row>
@@ -1766,9 +1771,9 @@
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659071023</t>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframedgrameen-a-village-scene</t>
         </is>
       </c>
     </row>
@@ -1795,9 +1800,9 @@
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496656089135</t>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframed-sita-swayamvar</t>
         </is>
       </c>
     </row>
@@ -1824,9 +1829,9 @@
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641736751</t>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/dashavtaar-11-by-30</t>
         </is>
       </c>
     </row>
@@ -1853,9 +1858,9 @@
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649502767</t>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/durga-parivar-48-by-29</t>
         </is>
       </c>
     </row>
@@ -1882,9 +1887,9 @@
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496655007791</t>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hanuman-chalisa</t>
         </is>
       </c>
     </row>
@@ -1911,9 +1916,9 @@
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649633839</t>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/error</t>
         </is>
       </c>
     </row>
@@ -1940,9 +1945,9 @@
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641572911</t>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-kali-22-by-30-bharni-style</t>
         </is>
       </c>
     </row>
@@ -1969,9 +1974,9 @@
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649732143</t>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-lakshmi-22-5-by-7</t>
         </is>
       </c>
     </row>
@@ -1998,9 +2003,9 @@
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649699375</t>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-saraswati-11-by-14</t>
         </is>
       </c>
     </row>
@@ -2027,9 +2032,9 @@
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649666607</t>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/mahishashur-mardini-maa-durga</t>
         </is>
       </c>
     </row>
@@ -2056,9 +2061,9 @@
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641540143</t>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/mahishasur-mardini-22-by-30-madhubani-kachni-style</t>
         </is>
       </c>
     </row>
@@ -2085,9 +2090,9 @@
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649601071</t>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/raas-leela-24-by-29</t>
         </is>
       </c>
     </row>
@@ -2114,9 +2119,9 @@
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641802287</t>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/ram-sita-vivah-11-5-by-30-5</t>
         </is>
       </c>
     </row>
@@ -2143,9 +2148,9 @@
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496634069039</t>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/black-bishnupur-silk-dupatta-with-kantha-embroidery</t>
         </is>
       </c>
     </row>
@@ -2172,9 +2177,9 @@
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496658120751</t>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/black-linen-hand-embroidered-sujani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2201,9 +2206,9 @@
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496637378607</t>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/blue-hand-emdroidered-cotton-dupatta-with-hand-embroidered-kantha-jaal-work</t>
         </is>
       </c>
     </row>
@@ -2230,9 +2235,9 @@
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651403311</t>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/brown-linen-jamdani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2259,9 +2264,9 @@
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659628079</t>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-pure-raw-silk-dupatta-with-ghicha-tussar-edges</t>
         </is>
       </c>
     </row>
@@ -2288,9 +2293,9 @@
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659693615</t>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-pure-raw-silk-dupatta-with-ghicha-tussar-edges-1</t>
         </is>
       </c>
     </row>
@@ -2317,9 +2322,9 @@
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649994287</t>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-indigo-jamdani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2346,9 +2351,9 @@
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650092591</t>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-indigo-jamdani-dupatta-1</t>
         </is>
       </c>
     </row>
@@ -2375,9 +2380,9 @@
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650944559</t>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-cotton-dupatta-with-hand-embroidered-jamdani-motifs</t>
         </is>
       </c>
     </row>
@@ -2404,9 +2409,9 @@
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650059823</t>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-cotton-jamdani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2433,9 +2438,9 @@
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649895983</t>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-maroon-jamdani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2462,9 +2467,9 @@
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr"/>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649764911</t>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-plum-cotton-jamdani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2491,9 +2496,9 @@
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649830447</t>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-plum-cotton-jamdani-dupatta-1</t>
         </is>
       </c>
     </row>
@@ -2520,9 +2525,9 @@
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649928751</t>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-plum-teal-jamdani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2549,9 +2554,9 @@
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496649863215</t>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-teal-jamdani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2578,9 +2583,9 @@
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496640852015</t>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kantha-silk-dupatta</t>
         </is>
       </c>
     </row>
@@ -2607,9 +2612,9 @@
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651305007</t>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-dupatta-fulia-pink-with-blue-border</t>
         </is>
       </c>
     </row>
@@ -2640,9 +2645,9 @@
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651141167</t>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-shibori-dupatta</t>
         </is>
       </c>
     </row>
@@ -2673,9 +2678,9 @@
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651141167</t>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-shibori-dupatta</t>
         </is>
       </c>
     </row>
@@ -2702,9 +2707,9 @@
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496640720943</t>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-tussar-color-tree-of-life-dupatta</t>
         </is>
       </c>
     </row>
@@ -2731,9 +2736,9 @@
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496635707439</t>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-color-tussar-dupatta-with-hand-embroidered-kantha-work</t>
         </is>
       </c>
     </row>
@@ -2760,9 +2765,9 @@
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496635805743</t>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-color-tussar-dupatta-with-hand-embroidered-kantha-work-1</t>
         </is>
       </c>
     </row>
@@ -2789,9 +2794,9 @@
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496637345839</t>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-color-tussar-dupatta-with-hand-embroidered-kantha-work-2</t>
         </is>
       </c>
     </row>
@@ -2818,9 +2823,9 @@
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496633970735</t>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/peacock-blue-bishnupur-silk-dupatta-with-kantha-embroidery</t>
         </is>
       </c>
     </row>
@@ -2847,9 +2852,9 @@
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496656121903</t>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-chanderi-hand-embroidered-sujani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2876,9 +2881,9 @@
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496656220207</t>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta</t>
         </is>
       </c>
     </row>
@@ -2905,9 +2910,9 @@
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496656252975</t>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta-1</t>
         </is>
       </c>
     </row>
@@ -2934,9 +2939,9 @@
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr"/>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496656285743</t>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta-2</t>
         </is>
       </c>
     </row>
@@ -2963,9 +2968,9 @@
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496656351279</t>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta-3</t>
         </is>
       </c>
     </row>
@@ -2992,9 +2997,9 @@
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496636690479</t>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/salmon-pink-tussar-dupatta-with-hand-embroidered-kantha-work</t>
         </is>
       </c>
     </row>
@@ -3025,9 +3030,9 @@
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651730991</t>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/silk-cotton-baluchari-dupatta</t>
         </is>
       </c>
     </row>
@@ -3058,9 +3063,9 @@
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr"/>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651730991</t>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/silk-cotton-baluchari-dupatta</t>
         </is>
       </c>
     </row>
@@ -3087,9 +3092,9 @@
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496635838511</t>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/slate-grey-kutch-work-dupatta-on-hand-woven-tussar</t>
         </is>
       </c>
     </row>
@@ -3116,9 +3121,9 @@
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496633708591</t>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/teal-green-handwoven-cotton-moirang-phee-dupatta</t>
         </is>
       </c>
     </row>
@@ -3145,9 +3150,9 @@
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496658153519</t>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/yellow-bhagalpur-silk-hand-embroidered-sujani-dupatta</t>
         </is>
       </c>
     </row>
@@ -3174,9 +3179,9 @@
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr"/>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651501615</t>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/baluchari-unstitched-kurta-dupatta-set-magenta-on-off-white</t>
         </is>
       </c>
     </row>
@@ -3203,9 +3208,9 @@
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651567151</t>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/jamdani-cotton-unstitched-kurta-dupatta-set-black</t>
         </is>
       </c>
     </row>
@@ -3232,9 +3237,9 @@
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651665455</t>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/jamdani-cotton-unstitched-kurta-dupatta-set-taupe</t>
         </is>
       </c>
     </row>
@@ -3261,9 +3266,9 @@
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr"/>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496637476911</t>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tree-of-life-kantha-hand-embroidered-bishnupur-silk-dress-material-2-5m</t>
         </is>
       </c>
     </row>
@@ -3290,9 +3295,9 @@
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496646389807</t>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-mekhala-chador-from-assam-1</t>
         </is>
       </c>
     </row>
@@ -3319,9 +3324,9 @@
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496646651951</t>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-mekhala-chador-from-assam-3</t>
         </is>
       </c>
     </row>
@@ -3348,9 +3353,9 @@
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651698223</t>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/corn-flower-blue-matka-baluchari-stole</t>
         </is>
       </c>
     </row>
@@ -3377,9 +3382,9 @@
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496640917551</t>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cotton-silk-stole-with-black-hand-embroidered-kantha-work</t>
         </is>
       </c>
     </row>
@@ -3406,9 +3411,9 @@
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496633905199</t>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cotton-silk-stole-with-hand-embroidered-turquoise-kantha-work</t>
         </is>
       </c>
     </row>
@@ -3435,9 +3440,9 @@
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr"/>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650125359</t>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/dhanekhali-stole</t>
         </is>
       </c>
     </row>
@@ -3464,9 +3469,9 @@
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr"/>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496641114159</t>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-kantha-on-two-toned-handwoven-silk</t>
         </is>
       </c>
     </row>
@@ -3493,9 +3498,9 @@
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr"/>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496640983087</t>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-nakshi-kantha-on-handwoven-silk</t>
         </is>
       </c>
     </row>
@@ -3522,9 +3527,9 @@
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr"/>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496655466543</t>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-sujani-stole</t>
         </is>
       </c>
     </row>
@@ -3551,9 +3556,9 @@
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr"/>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496655532079</t>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-sujani-stole-1</t>
         </is>
       </c>
     </row>
@@ -3580,9 +3585,9 @@
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr"/>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496655597615</t>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/intricately-hand-embroidered-silk-stole</t>
         </is>
       </c>
     </row>
@@ -3613,9 +3618,9 @@
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr"/>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650584111</t>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-cotton-silk-stole-with-extra-weft-motifs</t>
         </is>
       </c>
     </row>
@@ -3646,9 +3651,9 @@
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr"/>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650584111</t>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-cotton-silk-stole-with-extra-weft-motifs</t>
         </is>
       </c>
     </row>
@@ -3675,9 +3680,9 @@
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr"/>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659595311</t>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tone-on-tone-handwoven-grey-tussar-stole-with-sujani-hand-embroidery</t>
         </is>
       </c>
     </row>
@@ -3704,9 +3709,9 @@
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr"/>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650354735</t>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-black-and-white-cotton-jamdani-stole</t>
         </is>
       </c>
     </row>
@@ -3733,9 +3738,9 @@
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr"/>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650846255</t>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-cotton-jamdani-stole-with-cute-tassels</t>
         </is>
       </c>
     </row>
@@ -3762,9 +3767,9 @@
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr"/>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650453039</t>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-red-and-off-white-cotton-jamdani-stole</t>
         </is>
       </c>
     </row>
@@ -3791,9 +3796,9 @@
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr"/>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650518575</t>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/lilac-cotton-jamdani-stole</t>
         </is>
       </c>
     </row>
@@ -3820,9 +3825,9 @@
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr"/>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651075631</t>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-stole-with-extra-weft-motifs</t>
         </is>
       </c>
     </row>
@@ -3853,9 +3858,9 @@
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr"/>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651010095</t>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-stole-with-jaquard-hand-woven-motifs</t>
         </is>
       </c>
     </row>
@@ -3882,9 +3887,9 @@
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr"/>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650190895</t>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/olive-handwoven-cotton-jamdani-stole</t>
         </is>
       </c>
     </row>
@@ -3911,9 +3916,9 @@
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr"/>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496651436079</t>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/pink-linen-jamdani-stole</t>
         </is>
       </c>
     </row>
@@ -3940,9 +3945,9 @@
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr"/>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496650977327</t>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-handwoven-matka-silk-stole-with-zari-stripes</t>
         </is>
       </c>
     </row>
@@ -3969,9 +3974,9 @@
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr"/>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496633937967</t>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/reversible-pure-silk-hand-embroidered-kantha-stole</t>
         </is>
       </c>
     </row>
@@ -3998,13 +4003,133 @@
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr"/>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496658284591</t>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-stole</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="rId118"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weights sheet: update Maa Kali link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GZ6mf45gFCeDpGL3ireK6C
</commit_message>
<xml_diff>
--- a/docs/Bhoomija_Weights_Needed.xlsx
+++ b/docs/Bhoomija_Weights_Needed.xlsx
@@ -499,7 +499,6 @@
           <t>Hand embroidered Kauna U Bag</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>ACC-BAG-0001</t>
@@ -528,7 +527,6 @@
           <t>Hand embroidered U bag</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>ACC-BAG-0003</t>
@@ -557,7 +555,6 @@
           <t>Hand embroidered bag</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>ACC-BAG-0004</t>
@@ -586,7 +583,6 @@
           <t>Hand embroidered water hyacinth bag</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>ACC-BAG-0002</t>
@@ -615,7 +611,6 @@
           <t>Kauna Cherry bag with Bhoomija logo</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>ACC-BAG-0005</t>
@@ -644,7 +639,6 @@
           <t>Naga Belt (Brown)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>ACC-BLT-0001</t>
@@ -1036,7 +1030,6 @@
           <t>Kauna Purse White Flower with Green leaves</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>ACC-CLT-0001</t>
@@ -1230,7 +1223,6 @@
           <t>Plain Moon Clutch (Waterhyacinth)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>ACC-CLT-0004</t>
@@ -1259,7 +1251,6 @@
           <t>Water hyacinth handbag</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>GBC-BAG-0001</t>
@@ -1387,7 +1378,6 @@
           <t>Sujani hand embroidered Wall hanger - Sujani embroidery in process</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>GHA-WHG-0004</t>
@@ -1416,7 +1406,6 @@
           <t>Bawan Buti Bedspread -Single</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>HOM-BSP-0007</t>
@@ -1445,7 +1434,6 @@
           <t>Bawan Buti Bedspread -Single</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>HOM-BSP-0008</t>
@@ -1474,7 +1462,6 @@
           <t>Bawan Buti Bedspread -Single</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>HOM-BSP-0009</t>
@@ -1503,7 +1490,6 @@
           <t>Bawan Buti Bedspread -Single</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>HOM-BSP-0010</t>
@@ -1532,7 +1518,6 @@
           <t>Bawan Buti Bedspread -Single</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>HOM-BSP-0011</t>
@@ -1561,7 +1546,6 @@
           <t>Bawan Buti Bedspread -Single</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>HOM-BSP-0012</t>
@@ -1590,7 +1574,6 @@
           <t>Bawan Buti cotton Bedspread- king</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>HOM-BSP-0001</t>
@@ -1619,7 +1602,6 @@
           <t>Bawan Buti cotton Bedspread- king</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>HOM-BSP-0002</t>
@@ -1648,7 +1630,6 @@
           <t>Bawan Buti cotton Bedspread- king</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>HOM-BSP-0003</t>
@@ -1677,7 +1658,6 @@
           <t>Bawan Buti cotton bed spread - queen</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>HOM-BSP-0004</t>
@@ -1706,7 +1686,6 @@
           <t>Bawan Buti cotton bed spread - queen</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>HOM-BSP-0005</t>
@@ -1735,7 +1714,6 @@
           <t>Bawan Buti cotton bed spread - queen</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>HOM-BSP-0006</t>
@@ -1764,7 +1742,6 @@
           <t>Sujani hand embroidered Wall hanger - Grameen</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>WAR-EWH-0004</t>
@@ -1793,7 +1770,6 @@
           <t>Sujani hand embroidered Wall hanger - Sita Swayamvar</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>WAR-EWH-0003</t>
@@ -1822,7 +1798,6 @@
           <t>Dashavtaar Madhubani Art</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>WAR-PNT-0003</t>
@@ -1851,7 +1826,6 @@
           <t>Durga Parivar - Kalighat Painting</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>WAR-PNT-0005</t>
@@ -1880,7 +1854,6 @@
           <t>Hanuman Chalisa Madhubani Art</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>WAR-PNT-0011</t>
@@ -1909,7 +1882,6 @@
           <t>Maa Kali - Kalighat Painting</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>WAR-PNT-0007</t>
@@ -1918,7 +1890,7 @@
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>https://bhoomija.in/products/error</t>
+          <t>https://bhoomija.in/products/maa-kali-28-by-22</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1910,6 @@
           <t>Maa Kali Madhubani Art</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>WAR-PNT-0002</t>
@@ -1967,7 +1938,6 @@
           <t>Maa Lakshmi - Kalighat Painting</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>WAR-PNT-0010</t>
@@ -1996,7 +1966,6 @@
           <t>Maa Saraswati - Kalighat Painting</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>WAR-PNT-0009</t>
@@ -2025,7 +1994,6 @@
           <t>Mahishasur Mardini Maa Durga - Kalighat Painting</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>WAR-PNT-0008</t>
@@ -2054,7 +2022,6 @@
           <t>Mahishasur Mardini Madhubani Art</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>WAR-PNT-0001</t>
@@ -2083,7 +2050,6 @@
           <t>Raas Leela - Kalighat Painting</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>WAR-PNT-0006</t>
@@ -2112,7 +2078,6 @@
           <t>Ram Sita Vivah Madhubani Art</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>WAR-PNT-0004</t>
@@ -2141,7 +2106,6 @@
           <t>Black Bishnupur silk dupatta with Kantha embroidery</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>WEA-DUP-0003</t>
@@ -2170,7 +2134,6 @@
           <t>Black linen hand embroidered Sujani dupatta</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>WEA-DUP-0030</t>
@@ -2199,7 +2162,6 @@
           <t>Blue hand embroidered cotton dupatta with hand embroidered Kantha jaal work</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>WEA-DUP-0009</t>
@@ -2228,7 +2190,6 @@
           <t>Brown Linen Jamdani dupatta</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>WEA-DUP-0023</t>
@@ -2257,7 +2218,6 @@
           <t>Hand woven pure raw silk dupatta with ghicha tussar edges</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>WEA-DUP-0032</t>
@@ -2286,7 +2246,6 @@
           <t>Hand woven pure raw silk dupatta with ghicha tussar edges</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>WEA-DUP-0033</t>
@@ -2315,7 +2274,6 @@
           <t>Handwoven Indigo jamdani dupatta</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>WEA-DUP-0017</t>
@@ -2344,7 +2302,6 @@
           <t>Handwoven Indigo jamdani dupatta</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>WEA-DUP-0019</t>
@@ -2373,7 +2330,6 @@
           <t>Handwoven cotton dupatta with hand embroidered jamdani motifs</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>WEA-DUP-0020</t>
@@ -2402,7 +2358,6 @@
           <t>Handwoven cotton jamdani dupatta</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>WEA-DUP-0018</t>
@@ -2431,7 +2386,6 @@
           <t>Handwoven maroon jamdani dupatta</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>WEA-DUP-0015</t>
@@ -2460,7 +2414,6 @@
           <t>Handwoven plum cotton jamdani dupatta</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
           <t>WEA-DUP-0012</t>
@@ -2489,7 +2442,6 @@
           <t>Handwoven plum cotton jamdani dupatta</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
           <t>WEA-DUP-0013</t>
@@ -2518,7 +2470,6 @@
           <t>Handwoven plum teal jamdani dupatta</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
           <t>WEA-DUP-0016</t>
@@ -2547,7 +2498,6 @@
           <t>Handwoven teal jamdani dupatta</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
           <t>WEA-DUP-0014</t>
@@ -2576,7 +2526,6 @@
           <t>Kantha silk dupatta</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>WEA-DUP-0011</t>
@@ -2605,7 +2554,6 @@
           <t>Matka Silk Dupatta Fulia (Pink with Blue border)</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
           <t>WEA-DUP-0022</t>
@@ -2700,7 +2648,6 @@
           <t>Natural Tussar color tree of life dupatta</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>WEA-DUP-0010</t>
@@ -2729,7 +2676,6 @@
           <t>Natural color tussar dupatta with hand embroidered Kantha work</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>WEA-DUP-0004</t>
@@ -2758,7 +2704,6 @@
           <t>Natural color tussar dupatta with hand embroidered Kantha work</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>WEA-DUP-0005</t>
@@ -2787,7 +2732,6 @@
           <t>Natural color tussar dupatta with hand embroidered Kantha work</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>WEA-DUP-0008</t>
@@ -2816,7 +2760,6 @@
           <t>Peacock Blue Bishnupur Silk dupatta with Kantha embroidery</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>WEA-DUP-0002</t>
@@ -2845,7 +2788,6 @@
           <t>Red chanderi hand embroidered Sujani dupatta</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>WEA-DUP-0025</t>
@@ -2874,7 +2816,6 @@
           <t>Red linen hand embroidered Sujani dupatta</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>WEA-DUP-0026</t>
@@ -2903,7 +2844,6 @@
           <t>Red linen hand embroidered Sujani dupatta</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>WEA-DUP-0027</t>
@@ -2932,7 +2872,6 @@
           <t>Red linen hand embroidered Sujani dupatta</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>WEA-DUP-0028</t>
@@ -2961,7 +2900,6 @@
           <t>Red linen hand embroidered Sujani dupatta</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
           <t>WEA-DUP-0029</t>
@@ -2990,7 +2928,6 @@
           <t>Salmon pink tussar dupatta with hand embroidered Kantha work</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>WEA-DUP-0007</t>
@@ -3085,7 +3022,6 @@
           <t>Slate grey Kutch work dupatta on hand woven tussar</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>WEA-DUP-0006</t>
@@ -3114,7 +3050,6 @@
           <t>Teal green handwoven cotton Moirang Phee dupatta</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>WEA-DUP-0001</t>
@@ -3143,7 +3078,6 @@
           <t>Yellow Bhagalpur silk hand embroidered Sujani dupatta</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>WEA-DUP-0031</t>
@@ -3172,7 +3106,6 @@
           <t>Baluchari Unstitched Kurta Dupatta set (Magenta on Off White)</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
           <t>WEA-FAB-0002</t>
@@ -3201,7 +3134,6 @@
           <t>Jamdani Cotton Unstitched Kurta Dupatta set (Black)</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
           <t>WEA-FAB-0003</t>
@@ -3230,7 +3162,6 @@
           <t>Jamdani Cotton Unstitched Kurta Dupatta set (Taupe)</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>WEA-FAB-0004</t>
@@ -3259,7 +3190,6 @@
           <t>Tree of life kantha hand embroidered Bishnupur silk dress material 2.5m</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
           <t>WEA-FAB-0001</t>
@@ -3288,7 +3218,6 @@
           <t>Handwoven Mekhala Chador from Assam</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>WEA-MKC-0002</t>
@@ -3317,7 +3246,6 @@
           <t>Handwoven Mekhala Chador from Assam</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>WEA-MKC-0004</t>
@@ -3346,7 +3274,6 @@
           <t>Corn flower blue Matka Baluchari Stole</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
         <is>
           <t>WEA-STL-0020</t>
@@ -3375,7 +3302,6 @@
           <t>Cotton silk stole with black hand embroidered kantha work</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>WEA-STL-0004</t>
@@ -3404,7 +3330,6 @@
           <t>Cotton silk stole with hand embroidered turquoise Kantha work</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>WEA-STL-0002</t>
@@ -3433,7 +3358,6 @@
           <t>Dhanekhali Stole</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>WEA-STL-0009</t>
@@ -3462,7 +3386,6 @@
           <t>Hand embroidered Kantha on two toned handwoven silk</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>WEA-STL-0006</t>
@@ -3491,7 +3414,6 @@
           <t>Hand embroidered Nakshi Kantha on handwoven silk</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
         <is>
           <t>WEA-STL-0005</t>
@@ -3520,7 +3442,6 @@
           <t>Hand embroidered Sujani stole</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
           <t>WEA-STL-0021</t>
@@ -3549,7 +3470,6 @@
           <t>Hand embroidered Sujani stole</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>WEA-STL-0022</t>
@@ -3578,7 +3498,6 @@
           <t>Hand embroidered Sujani stole - Cream with intricacies</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
           <t>WEA-STL-0023</t>
@@ -3673,7 +3592,6 @@
           <t>Handwoven Grey tussar stole with Sujani hand embroidery.</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>WEA-STL-0025</t>
@@ -3702,7 +3620,6 @@
           <t>Handwoven black and white cotton jamdani stole</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
           <t>WEA-STL-0011</t>
@@ -3731,7 +3648,6 @@
           <t>Handwoven cotton jamdani stole with cute tassels</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
           <t>WEA-STL-0015</t>
@@ -3760,7 +3676,6 @@
           <t>Handwoven red and off white cotton jamdani stole</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
           <t>WEA-STL-0012</t>
@@ -3789,7 +3704,6 @@
           <t>Lilac cotton jamdani stole</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
         <is>
           <t>WEA-STL-0013</t>
@@ -3818,7 +3732,6 @@
           <t>Matka Silk Stole with extra weft motifs</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
           <t>WEA-STL-0018</t>
@@ -3880,7 +3793,6 @@
           <t>Olive handwoven cotton jamdani stole</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
           <t>WEA-STL-0010</t>
@@ -3909,7 +3821,6 @@
           <t>Pink linen Jamdani stole</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
           <t>WEA-STL-0019</t>
@@ -3938,7 +3849,6 @@
           <t>Red handwoven Matka Silk stole with zari stripes</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
           <t>WEA-STL-0016</t>
@@ -3967,7 +3877,6 @@
           <t>Reversible pure silk hand embroidered Kantha stole</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr">
         <is>
           <t>WEA-STL-0003</t>
@@ -3996,7 +3905,6 @@
           <t>Sujani Stole - Beige</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
           <t>WEA-STL-0024</t>

</xml_diff>